<commit_message>
try to fix set ell accounting US Dollar, not finished yet
</commit_message>
<xml_diff>
--- a/2-Tests/OpenExcelSdk.Tests/10-Files/SetCellValueCurrency.xlsx
+++ b/2-Tests/OpenExcelSdk.Tests/10-Files/SetCellValueCurrency.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/OpenExcelSdk/Dev/OpenExcelSdk/2-Tests/OpenExcelSdk.Tests/10-Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="209" documentId="11_AD4DB114E441178AC67DF4536695FF58683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57F3795E-B71E-4DE3-86FB-53F72992BF05}"/>
+  <xr:revisionPtr revIDLastSave="237" documentId="11_AD4DB114E441178AC67DF4536695FF58683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{116EB83F-D083-4446-9503-9A71905C8F1E}"/>
   <bookViews>
-    <workbookView xWindow="7350" yWindow="3285" windowWidth="21075" windowHeight="13350" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9300" yWindow="5925" windowWidth="18885" windowHeight="11355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="11">
   <si>
     <t>value</t>
   </si>
@@ -36,32 +36,36 @@
     <t>info</t>
   </si>
   <si>
-    <t>accounting, 456,89; USD</t>
-  </si>
-  <si>
-    <t>currency, 456,89; USD</t>
-  </si>
-  <si>
-    <t>accouting; euro</t>
-  </si>
-  <si>
-    <t>currency;euro</t>
-  </si>
-  <si>
-    <t>currency; euro</t>
-  </si>
-  <si>
-    <t>currency;euro; red, no neg sign</t>
-  </si>
-  <si>
-    <t>currency;euro; red</t>
+    <t>currency</t>
+  </si>
+  <si>
+    <t>euro</t>
+  </si>
+  <si>
+    <t>accounting</t>
+  </si>
+  <si>
+    <t>currency; leftSpace</t>
+  </si>
+  <si>
+    <t>currency;RedNeg;NoSign</t>
+  </si>
+  <si>
+    <t>currency;RedNeg</t>
+  </si>
+  <si>
+    <t>US Dollar</t>
+  </si>
+  <si>
+    <t>Swiss Franc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="7">
+  <numFmts count="8">
+    <numFmt numFmtId="7" formatCode="#,##0.00\ &quot;€&quot;;\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ hh:mm:ss"/>
@@ -113,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -123,6 +127,7 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="7" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -407,13 +412,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.42578125" customWidth="1"/>
     <col min="2" max="2" width="22.5703125" customWidth="1"/>
     <col min="3" max="3" width="20.85546875" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" customWidth="1"/>
+    <col min="4" max="4" width="32.140625" customWidth="1"/>
     <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -427,71 +432,124 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="3">
-        <v>123</v>
+        <v>5</v>
+      </c>
+      <c r="C2" s="6">
+        <v>-12.34</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C3" s="3">
         <v>-392.78</v>
       </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="7">
+        <v>6</v>
+      </c>
+      <c r="C4" s="9">
         <v>-550</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="8">
-        <v>-988</v>
+        <v>7</v>
+      </c>
+      <c r="C5" s="7">
+        <v>-71</v>
+      </c>
+      <c r="D5" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="6">
-        <v>-8900</v>
+        <v>8</v>
+      </c>
+      <c r="C6" s="8">
+        <v>-62</v>
+      </c>
+      <c r="D6" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C7" s="6"/>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C8" s="6"/>
+      <c r="D8" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="4">
-        <v>456.89</v>
+      <c r="C9" s="4"/>
+      <c r="D9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="5">
-        <v>678.34</v>
+      <c r="C10" s="5"/>
+      <c r="D10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>10</v>
+      </c>
       <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D17" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
pb SetCellValue accounting US-dollar fixed
</commit_message>
<xml_diff>
--- a/2-Tests/OpenExcelSdk.Tests/10-Files/SetCellValueCurrency.xlsx
+++ b/2-Tests/OpenExcelSdk.Tests/10-Files/SetCellValueCurrency.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/OpenExcelSdk/Dev/OpenExcelSdk/2-Tests/OpenExcelSdk.Tests/10-Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="237" documentId="11_AD4DB114E441178AC67DF4536695FF58683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{116EB83F-D083-4446-9503-9A71905C8F1E}"/>
+  <xr:revisionPtr revIDLastSave="250" documentId="11_AD4DB114E441178AC67DF4536695FF58683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{753E55AF-A384-4A56-8800-D342A64A6935}"/>
   <bookViews>
-    <workbookView xWindow="9300" yWindow="5925" windowWidth="18885" windowHeight="11355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6960" yWindow="1950" windowWidth="19110" windowHeight="13830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="11">
   <si>
     <t>value</t>
   </si>
@@ -64,7 +64,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="8">
+  <numFmts count="16">
     <numFmt numFmtId="7" formatCode="#,##0.00\ &quot;€&quot;;\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
@@ -73,6 +73,14 @@
     <numFmt numFmtId="166" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
     <numFmt numFmtId="167" formatCode="[$$-409]#,##0.00"/>
     <numFmt numFmtId="168" formatCode="#,##0.00\ &quot;€&quot;;[Red]#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="169" formatCode="[$$-409]#,##0.00_ ;\-[$$-409]#,##0.00\ "/>
+    <numFmt numFmtId="170" formatCode="[$$-409]#,##0.00;[Red][$$-409]#,##0.00"/>
+    <numFmt numFmtId="171" formatCode="[$$-409]#,##0.00_ ;[Red]\-[$$-409]#,##0.00\ "/>
+    <numFmt numFmtId="172" formatCode="_-* #,##0.00\ [$CHF-100C]_-;\-* #,##0.00\ [$CHF-100C]_-;_-* &quot;-&quot;??\ [$CHF-100C]_-;_-@_-"/>
+    <numFmt numFmtId="173" formatCode="#,##0.00\ [$CHF-100C]"/>
+    <numFmt numFmtId="174" formatCode="#,##0.00\ [$CHF-100C];\-#,##0.00\ [$CHF-100C]"/>
+    <numFmt numFmtId="175" formatCode="#,##0.00\ [$CHF-100C];[Red]#,##0.00\ [$CHF-100C]"/>
+    <numFmt numFmtId="176" formatCode="#,##0.00\ [$CHF-100C];[Red]\-#,##0.00\ [$CHF-100C]"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -117,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -128,6 +136,14 @@
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="7" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -412,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.42578125" customWidth="1"/>
@@ -492,62 +508,83 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C7" s="6"/>
+      <c r="C7" s="4">
+        <v>-12.34</v>
+      </c>
       <c r="D7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C8" s="6"/>
+      <c r="C8" s="5">
+        <v>-392.78</v>
+      </c>
       <c r="D8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C9" s="4"/>
+      <c r="C9" s="10">
+        <v>-550</v>
+      </c>
       <c r="D9" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C10" s="5"/>
+      <c r="C10" s="11">
+        <v>-71</v>
+      </c>
       <c r="D10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C11" s="12">
+        <v>-62</v>
+      </c>
       <c r="D11" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C12" s="13">
+        <v>-12.34</v>
+      </c>
       <c r="D12" t="s">
         <v>10</v>
       </c>
       <c r="F12" s="3"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C13" s="14">
+        <v>-392.78</v>
+      </c>
       <c r="D13" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C14" s="15">
+        <v>-550</v>
+      </c>
       <c r="D14" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C15" s="16">
+        <v>-71</v>
+      </c>
       <c r="D15" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C16" s="17">
+        <v>-62</v>
+      </c>
       <c r="D16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D17" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>